<commit_message>
All LF results computed
</commit_message>
<xml_diff>
--- a/Step4_Snorkel_Results.xlsx
+++ b/Step4_Snorkel_Results.xlsx
@@ -10463,8 +10463,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+  <fonts count="5">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -10513,7 +10521,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -10521,19 +10529,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -10833,166 +10859,166 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:54">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>53</v>
       </c>
     </row>
@@ -11018,7 +11044,7 @@
       <c r="G2" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I2">
@@ -11182,7 +11208,7 @@
       <c r="G3" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I3">
@@ -11346,7 +11372,7 @@
       <c r="G4" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I4">
@@ -11510,7 +11536,7 @@
       <c r="G5" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I5">
@@ -11674,7 +11700,7 @@
       <c r="G6" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I6">
@@ -11838,7 +11864,7 @@
       <c r="G7" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I7">
@@ -12002,7 +12028,7 @@
       <c r="G8" t="s">
         <v>3</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I8">
@@ -12166,7 +12192,7 @@
       <c r="G9" t="s">
         <v>3</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I9">
@@ -12330,7 +12356,7 @@
       <c r="G10" t="s">
         <v>3</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I10">
@@ -12494,7 +12520,7 @@
       <c r="G11" t="s">
         <v>5</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I11">
@@ -12658,7 +12684,7 @@
       <c r="G12" t="s">
         <v>3</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I12">
@@ -12822,7 +12848,7 @@
       <c r="G13" t="s">
         <v>5</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I13">
@@ -12986,7 +13012,7 @@
       <c r="G14" t="s">
         <v>4</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I14">
@@ -13150,7 +13176,7 @@
       <c r="G15" t="s">
         <v>3</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I15">
@@ -13314,7 +13340,7 @@
       <c r="G16" t="s">
         <v>5</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I16">
@@ -13478,7 +13504,7 @@
       <c r="G17" t="s">
         <v>4</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="H17" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I17">
@@ -13642,7 +13668,7 @@
       <c r="G18" t="s">
         <v>3</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="H18" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I18">
@@ -13806,7 +13832,7 @@
       <c r="G19" t="s">
         <v>3</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I19">
@@ -13970,7 +13996,7 @@
       <c r="G20" t="s">
         <v>3</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I20">
@@ -14134,7 +14160,7 @@
       <c r="G21" t="s">
         <v>4</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="H21" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I21">
@@ -14298,7 +14324,7 @@
       <c r="G22" t="s">
         <v>3</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I22">
@@ -14626,7 +14652,7 @@
       <c r="G24" t="s">
         <v>5</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="H24" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I24">
@@ -14790,7 +14816,7 @@
       <c r="G25" t="s">
         <v>3</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="H25" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I25">
@@ -14954,7 +14980,7 @@
       <c r="G26" t="s">
         <v>3</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="H26" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I26">
@@ -15118,7 +15144,7 @@
       <c r="G27" t="s">
         <v>5</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="H27" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I27">
@@ -15282,7 +15308,7 @@
       <c r="G28" t="s">
         <v>3</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="H28" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I28">
@@ -15446,7 +15472,7 @@
       <c r="G29" t="s">
         <v>3</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="H29" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I29">
@@ -15610,7 +15636,7 @@
       <c r="G30" t="s">
         <v>3</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="H30" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I30">
@@ -15774,7 +15800,7 @@
       <c r="G31" t="s">
         <v>5</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="H31" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I31">
@@ -15938,7 +15964,7 @@
       <c r="G32" t="s">
         <v>4</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="H32" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I32">
@@ -16102,7 +16128,7 @@
       <c r="G33" t="s">
         <v>3</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="H33" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I33">
@@ -16251,7 +16277,7 @@
       <c r="B34" t="s">
         <v>385</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="4" t="s">
         <v>669</v>
       </c>
       <c r="D34">
@@ -16266,7 +16292,7 @@
       <c r="G34" t="s">
         <v>3</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="H34" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I34">
@@ -16412,10 +16438,10 @@
       <c r="A35" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="4" t="s">
         <v>386</v>
       </c>
       <c r="D35">
@@ -16430,7 +16456,7 @@
       <c r="G35" t="s">
         <v>3</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="H35" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I35">
@@ -16594,7 +16620,7 @@
       <c r="G36" t="s">
         <v>5</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H36" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I36">
@@ -16758,7 +16784,7 @@
       <c r="G37" t="s">
         <v>3</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="H37" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I37">
@@ -16922,7 +16948,7 @@
       <c r="G38" t="s">
         <v>5</v>
       </c>
-      <c r="H38" s="2" t="s">
+      <c r="H38" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I38">
@@ -17086,7 +17112,7 @@
       <c r="G39" t="s">
         <v>4</v>
       </c>
-      <c r="H39" s="1" t="s">
+      <c r="H39" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I39">
@@ -17250,7 +17276,7 @@
       <c r="G40" t="s">
         <v>5</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="H40" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I40">
@@ -17414,7 +17440,7 @@
       <c r="G41" t="s">
         <v>5</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="H41" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I41">
@@ -17578,7 +17604,7 @@
       <c r="G42" t="s">
         <v>4</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="H42" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I42">
@@ -17742,7 +17768,7 @@
       <c r="G43" t="s">
         <v>3</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="H43" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I43">
@@ -17906,7 +17932,7 @@
       <c r="G44" t="s">
         <v>5</v>
       </c>
-      <c r="H44" s="2" t="s">
+      <c r="H44" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I44">
@@ -18070,7 +18096,7 @@
       <c r="G45" t="s">
         <v>5</v>
       </c>
-      <c r="H45" s="1" t="s">
+      <c r="H45" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I45">
@@ -18234,7 +18260,7 @@
       <c r="G46" t="s">
         <v>3</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="H46" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I46">
@@ -18398,7 +18424,7 @@
       <c r="G47" t="s">
         <v>5</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="H47" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I47">
@@ -18562,7 +18588,7 @@
       <c r="G48" t="s">
         <v>5</v>
       </c>
-      <c r="H48" s="2" t="s">
+      <c r="H48" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I48">
@@ -18726,7 +18752,7 @@
       <c r="G49" t="s">
         <v>5</v>
       </c>
-      <c r="H49" s="1" t="s">
+      <c r="H49" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I49">
@@ -18890,7 +18916,7 @@
       <c r="G50" t="s">
         <v>3</v>
       </c>
-      <c r="H50" s="1" t="s">
+      <c r="H50" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I50">
@@ -19054,7 +19080,7 @@
       <c r="G51" t="s">
         <v>5</v>
       </c>
-      <c r="H51" s="1" t="s">
+      <c r="H51" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I51">
@@ -19218,7 +19244,7 @@
       <c r="G52" t="s">
         <v>3</v>
       </c>
-      <c r="H52" s="2" t="s">
+      <c r="H52" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I52">
@@ -19382,7 +19408,7 @@
       <c r="G53" t="s">
         <v>5</v>
       </c>
-      <c r="H53" s="1" t="s">
+      <c r="H53" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I53">
@@ -19546,7 +19572,7 @@
       <c r="G54" t="s">
         <v>5</v>
       </c>
-      <c r="H54" s="1" t="s">
+      <c r="H54" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I54">
@@ -19710,7 +19736,7 @@
       <c r="G55" t="s">
         <v>5</v>
       </c>
-      <c r="H55" s="2" t="s">
+      <c r="H55" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I55">
@@ -19874,7 +19900,7 @@
       <c r="G56" t="s">
         <v>5</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="H56" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I56">
@@ -20038,7 +20064,7 @@
       <c r="G57" t="s">
         <v>5</v>
       </c>
-      <c r="H57" s="1" t="s">
+      <c r="H57" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I57">
@@ -20202,7 +20228,7 @@
       <c r="G58" t="s">
         <v>4</v>
       </c>
-      <c r="H58" s="1" t="s">
+      <c r="H58" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I58">
@@ -20366,7 +20392,7 @@
       <c r="G59" t="s">
         <v>5</v>
       </c>
-      <c r="H59" s="1" t="s">
+      <c r="H59" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I59">
@@ -20530,7 +20556,7 @@
       <c r="G60" t="s">
         <v>5</v>
       </c>
-      <c r="H60" s="2" t="s">
+      <c r="H60" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I60">
@@ -20694,7 +20720,7 @@
       <c r="G61" t="s">
         <v>3</v>
       </c>
-      <c r="H61" s="1" t="s">
+      <c r="H61" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I61">
@@ -20858,7 +20884,7 @@
       <c r="G62" t="s">
         <v>5</v>
       </c>
-      <c r="H62" s="2" t="s">
+      <c r="H62" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I62">
@@ -21022,7 +21048,7 @@
       <c r="G63" t="s">
         <v>5</v>
       </c>
-      <c r="H63" s="1" t="s">
+      <c r="H63" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I63">
@@ -21186,7 +21212,7 @@
       <c r="G64" t="s">
         <v>5</v>
       </c>
-      <c r="H64" s="2" t="s">
+      <c r="H64" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I64">
@@ -21350,7 +21376,7 @@
       <c r="G65" t="s">
         <v>5</v>
       </c>
-      <c r="H65" s="2" t="s">
+      <c r="H65" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I65">
@@ -21514,7 +21540,7 @@
       <c r="G66" t="s">
         <v>5</v>
       </c>
-      <c r="H66" s="1" t="s">
+      <c r="H66" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I66">
@@ -21678,7 +21704,7 @@
       <c r="G67" t="s">
         <v>5</v>
       </c>
-      <c r="H67" s="1" t="s">
+      <c r="H67" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I67">
@@ -21842,7 +21868,7 @@
       <c r="G68" t="s">
         <v>3</v>
       </c>
-      <c r="H68" s="2" t="s">
+      <c r="H68" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I68">
@@ -22006,7 +22032,7 @@
       <c r="G69" t="s">
         <v>4</v>
       </c>
-      <c r="H69" s="1" t="s">
+      <c r="H69" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I69">
@@ -22170,7 +22196,7 @@
       <c r="G70" t="s">
         <v>3</v>
       </c>
-      <c r="H70" s="1" t="s">
+      <c r="H70" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I70">
@@ -22334,7 +22360,7 @@
       <c r="G71" t="s">
         <v>3</v>
       </c>
-      <c r="H71" s="2" t="s">
+      <c r="H71" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I71">
@@ -22498,7 +22524,7 @@
       <c r="G72" t="s">
         <v>3</v>
       </c>
-      <c r="H72" s="2" t="s">
+      <c r="H72" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I72">
@@ -22662,7 +22688,7 @@
       <c r="G73" t="s">
         <v>5</v>
       </c>
-      <c r="H73" s="2" t="s">
+      <c r="H73" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I73">
@@ -22826,7 +22852,7 @@
       <c r="G74" t="s">
         <v>3</v>
       </c>
-      <c r="H74" s="1" t="s">
+      <c r="H74" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I74">
@@ -22990,7 +23016,7 @@
       <c r="G75" t="s">
         <v>5</v>
       </c>
-      <c r="H75" s="1" t="s">
+      <c r="H75" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I75">
@@ -23154,7 +23180,7 @@
       <c r="G76" t="s">
         <v>4</v>
       </c>
-      <c r="H76" s="1" t="s">
+      <c r="H76" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I76">
@@ -23318,7 +23344,7 @@
       <c r="G77" t="s">
         <v>5</v>
       </c>
-      <c r="H77" s="2" t="s">
+      <c r="H77" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I77">
@@ -23482,7 +23508,7 @@
       <c r="G78" t="s">
         <v>5</v>
       </c>
-      <c r="H78" s="1" t="s">
+      <c r="H78" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I78">
@@ -23646,7 +23672,7 @@
       <c r="G79" t="s">
         <v>5</v>
       </c>
-      <c r="H79" s="1" t="s">
+      <c r="H79" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I79">
@@ -23810,7 +23836,7 @@
       <c r="G80" t="s">
         <v>5</v>
       </c>
-      <c r="H80" s="1" t="s">
+      <c r="H80" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I80">
@@ -23974,7 +24000,7 @@
       <c r="G81" t="s">
         <v>5</v>
       </c>
-      <c r="H81" s="1" t="s">
+      <c r="H81" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I81">
@@ -24138,7 +24164,7 @@
       <c r="G82" t="s">
         <v>5</v>
       </c>
-      <c r="H82" s="2" t="s">
+      <c r="H82" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I82">
@@ -24302,7 +24328,7 @@
       <c r="G83" t="s">
         <v>3</v>
       </c>
-      <c r="H83" s="2" t="s">
+      <c r="H83" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I83">
@@ -24466,7 +24492,7 @@
       <c r="G84" t="s">
         <v>4</v>
       </c>
-      <c r="H84" s="1" t="s">
+      <c r="H84" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I84">
@@ -24630,7 +24656,7 @@
       <c r="G85" t="s">
         <v>3</v>
       </c>
-      <c r="H85" s="2" t="s">
+      <c r="H85" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I85">
@@ -24794,7 +24820,7 @@
       <c r="G86" t="s">
         <v>5</v>
       </c>
-      <c r="H86" s="2" t="s">
+      <c r="H86" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I86">
@@ -24958,7 +24984,7 @@
       <c r="G87" t="s">
         <v>5</v>
       </c>
-      <c r="H87" s="1" t="s">
+      <c r="H87" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I87">
@@ -25122,7 +25148,7 @@
       <c r="G88" t="s">
         <v>4</v>
       </c>
-      <c r="H88" s="1" t="s">
+      <c r="H88" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I88">
@@ -25286,7 +25312,7 @@
       <c r="G89" t="s">
         <v>3</v>
       </c>
-      <c r="H89" s="2" t="s">
+      <c r="H89" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I89">
@@ -25450,7 +25476,7 @@
       <c r="G90" t="s">
         <v>3</v>
       </c>
-      <c r="H90" s="2" t="s">
+      <c r="H90" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I90">
@@ -25614,7 +25640,7 @@
       <c r="G91" t="s">
         <v>3</v>
       </c>
-      <c r="H91" s="2" t="s">
+      <c r="H91" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I91">
@@ -25778,7 +25804,7 @@
       <c r="G92" t="s">
         <v>3</v>
       </c>
-      <c r="H92" s="1" t="s">
+      <c r="H92" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I92">
@@ -25942,7 +25968,7 @@
       <c r="G93" t="s">
         <v>3</v>
       </c>
-      <c r="H93" s="1" t="s">
+      <c r="H93" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I93">
@@ -26106,7 +26132,7 @@
       <c r="G94" t="s">
         <v>5</v>
       </c>
-      <c r="H94" s="1" t="s">
+      <c r="H94" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I94">
@@ -26270,7 +26296,7 @@
       <c r="G95" t="s">
         <v>4</v>
       </c>
-      <c r="H95" s="1" t="s">
+      <c r="H95" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I95">
@@ -26434,7 +26460,7 @@
       <c r="G96" t="s">
         <v>3</v>
       </c>
-      <c r="H96" s="1" t="s">
+      <c r="H96" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I96">
@@ -26598,7 +26624,7 @@
       <c r="G97" t="s">
         <v>3</v>
       </c>
-      <c r="H97" s="2" t="s">
+      <c r="H97" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I97">
@@ -26762,7 +26788,7 @@
       <c r="G98" t="s">
         <v>5</v>
       </c>
-      <c r="H98" s="2" t="s">
+      <c r="H98" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I98">
@@ -26926,7 +26952,7 @@
       <c r="G99" t="s">
         <v>5</v>
       </c>
-      <c r="H99" s="1" t="s">
+      <c r="H99" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I99">
@@ -27090,7 +27116,7 @@
       <c r="G100" t="s">
         <v>5</v>
       </c>
-      <c r="H100" s="2" t="s">
+      <c r="H100" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I100">
@@ -27254,7 +27280,7 @@
       <c r="G101" t="s">
         <v>5</v>
       </c>
-      <c r="H101" s="1" t="s">
+      <c r="H101" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I101">
@@ -27418,7 +27444,7 @@
       <c r="G102" t="s">
         <v>3</v>
       </c>
-      <c r="H102" s="2" t="s">
+      <c r="H102" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I102">
@@ -27582,7 +27608,7 @@
       <c r="G103" t="s">
         <v>3</v>
       </c>
-      <c r="H103" s="1" t="s">
+      <c r="H103" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I103">
@@ -27746,7 +27772,7 @@
       <c r="G104" t="s">
         <v>3</v>
       </c>
-      <c r="H104" s="1" t="s">
+      <c r="H104" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I104">
@@ -27910,7 +27936,7 @@
       <c r="G105" t="s">
         <v>3</v>
       </c>
-      <c r="H105" s="1" t="s">
+      <c r="H105" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I105">
@@ -28074,7 +28100,7 @@
       <c r="G106" t="s">
         <v>3</v>
       </c>
-      <c r="H106" s="1" t="s">
+      <c r="H106" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I106">
@@ -28238,7 +28264,7 @@
       <c r="G107" t="s">
         <v>3</v>
       </c>
-      <c r="H107" s="2" t="s">
+      <c r="H107" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I107">
@@ -28402,7 +28428,7 @@
       <c r="G108" t="s">
         <v>5</v>
       </c>
-      <c r="H108" s="1" t="s">
+      <c r="H108" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I108">
@@ -28566,7 +28592,7 @@
       <c r="G109" t="s">
         <v>3</v>
       </c>
-      <c r="H109" s="2" t="s">
+      <c r="H109" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I109">
@@ -28730,7 +28756,7 @@
       <c r="G110" t="s">
         <v>5</v>
       </c>
-      <c r="H110" s="1" t="s">
+      <c r="H110" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I110">
@@ -28894,7 +28920,7 @@
       <c r="G111" t="s">
         <v>5</v>
       </c>
-      <c r="H111" s="2" t="s">
+      <c r="H111" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I111">
@@ -29058,7 +29084,7 @@
       <c r="G112" t="s">
         <v>3</v>
       </c>
-      <c r="H112" s="2" t="s">
+      <c r="H112" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I112">
@@ -29222,7 +29248,7 @@
       <c r="G113" t="s">
         <v>3</v>
       </c>
-      <c r="H113" s="2" t="s">
+      <c r="H113" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I113">
@@ -29386,7 +29412,7 @@
       <c r="G114" t="s">
         <v>3</v>
       </c>
-      <c r="H114" s="1" t="s">
+      <c r="H114" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I114">
@@ -29550,7 +29576,7 @@
       <c r="G115" t="s">
         <v>5</v>
       </c>
-      <c r="H115" s="1" t="s">
+      <c r="H115" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I115">
@@ -29714,7 +29740,7 @@
       <c r="G116" t="s">
         <v>3</v>
       </c>
-      <c r="H116" s="2" t="s">
+      <c r="H116" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I116">
@@ -29878,7 +29904,7 @@
       <c r="G117" t="s">
         <v>5</v>
       </c>
-      <c r="H117" s="2" t="s">
+      <c r="H117" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I117">
@@ -30042,7 +30068,7 @@
       <c r="G118" t="s">
         <v>5</v>
       </c>
-      <c r="H118" s="1" t="s">
+      <c r="H118" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I118">
@@ -30206,7 +30232,7 @@
       <c r="G119" t="s">
         <v>3</v>
       </c>
-      <c r="H119" s="1" t="s">
+      <c r="H119" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I119">
@@ -30370,7 +30396,7 @@
       <c r="G120" t="s">
         <v>5</v>
       </c>
-      <c r="H120" s="2" t="s">
+      <c r="H120" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I120">
@@ -30534,7 +30560,7 @@
       <c r="G121" t="s">
         <v>5</v>
       </c>
-      <c r="H121" s="1" t="s">
+      <c r="H121" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I121">
@@ -30698,7 +30724,7 @@
       <c r="G122" t="s">
         <v>5</v>
       </c>
-      <c r="H122" s="1" t="s">
+      <c r="H122" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I122">
@@ -30862,7 +30888,7 @@
       <c r="G123" t="s">
         <v>3</v>
       </c>
-      <c r="H123" s="2" t="s">
+      <c r="H123" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I123">
@@ -31026,7 +31052,7 @@
       <c r="G124" t="s">
         <v>3</v>
       </c>
-      <c r="H124" s="2" t="s">
+      <c r="H124" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I124">
@@ -31190,7 +31216,7 @@
       <c r="G125" t="s">
         <v>5</v>
       </c>
-      <c r="H125" s="1" t="s">
+      <c r="H125" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I125">
@@ -31354,7 +31380,7 @@
       <c r="G126" t="s">
         <v>3</v>
       </c>
-      <c r="H126" s="2" t="s">
+      <c r="H126" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I126">
@@ -31518,7 +31544,7 @@
       <c r="G127" t="s">
         <v>3</v>
       </c>
-      <c r="H127" s="2" t="s">
+      <c r="H127" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I127">
@@ -31682,7 +31708,7 @@
       <c r="G128" t="s">
         <v>3</v>
       </c>
-      <c r="H128" s="2" t="s">
+      <c r="H128" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I128">
@@ -31846,7 +31872,7 @@
       <c r="G129" t="s">
         <v>5</v>
       </c>
-      <c r="H129" s="2" t="s">
+      <c r="H129" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I129">
@@ -32010,7 +32036,7 @@
       <c r="G130" t="s">
         <v>5</v>
       </c>
-      <c r="H130" s="1" t="s">
+      <c r="H130" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I130">
@@ -32174,7 +32200,7 @@
       <c r="G131" t="s">
         <v>3</v>
       </c>
-      <c r="H131" s="2" t="s">
+      <c r="H131" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I131">
@@ -32338,7 +32364,7 @@
       <c r="G132" t="s">
         <v>3</v>
       </c>
-      <c r="H132" s="2" t="s">
+      <c r="H132" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I132">
@@ -32502,7 +32528,7 @@
       <c r="G133" t="s">
         <v>3</v>
       </c>
-      <c r="H133" s="2" t="s">
+      <c r="H133" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I133">
@@ -32666,7 +32692,7 @@
       <c r="G134" t="s">
         <v>3</v>
       </c>
-      <c r="H134" s="1" t="s">
+      <c r="H134" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I134">
@@ -32830,7 +32856,7 @@
       <c r="G135" t="s">
         <v>5</v>
       </c>
-      <c r="H135" s="2" t="s">
+      <c r="H135" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I135">
@@ -32994,7 +33020,7 @@
       <c r="G136" t="s">
         <v>3</v>
       </c>
-      <c r="H136" s="2" t="s">
+      <c r="H136" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I136">
@@ -33158,7 +33184,7 @@
       <c r="G137" t="s">
         <v>3</v>
       </c>
-      <c r="H137" s="2" t="s">
+      <c r="H137" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I137">
@@ -33322,7 +33348,7 @@
       <c r="G138" t="s">
         <v>5</v>
       </c>
-      <c r="H138" s="2" t="s">
+      <c r="H138" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I138">
@@ -33486,7 +33512,7 @@
       <c r="G139" t="s">
         <v>3</v>
       </c>
-      <c r="H139" s="2" t="s">
+      <c r="H139" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I139">
@@ -33650,7 +33676,7 @@
       <c r="G140" t="s">
         <v>3</v>
       </c>
-      <c r="H140" s="2" t="s">
+      <c r="H140" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I140">
@@ -33978,7 +34004,7 @@
       <c r="G142" t="s">
         <v>3</v>
       </c>
-      <c r="H142" s="2" t="s">
+      <c r="H142" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I142">
@@ -34142,7 +34168,7 @@
       <c r="G143" t="s">
         <v>5</v>
       </c>
-      <c r="H143" s="1" t="s">
+      <c r="H143" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I143">
@@ -34306,7 +34332,7 @@
       <c r="G144" t="s">
         <v>3</v>
       </c>
-      <c r="H144" s="2" t="s">
+      <c r="H144" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I144">
@@ -34470,7 +34496,7 @@
       <c r="G145" t="s">
         <v>3</v>
       </c>
-      <c r="H145" s="1" t="s">
+      <c r="H145" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I145">
@@ -34634,7 +34660,7 @@
       <c r="G146" t="s">
         <v>3</v>
       </c>
-      <c r="H146" s="2" t="s">
+      <c r="H146" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I146">
@@ -34798,7 +34824,7 @@
       <c r="G147" t="s">
         <v>4</v>
       </c>
-      <c r="H147" s="1" t="s">
+      <c r="H147" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I147">
@@ -34962,7 +34988,7 @@
       <c r="G148" t="s">
         <v>3</v>
       </c>
-      <c r="H148" s="2" t="s">
+      <c r="H148" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I148">
@@ -35126,7 +35152,7 @@
       <c r="G149" t="s">
         <v>5</v>
       </c>
-      <c r="H149" s="1" t="s">
+      <c r="H149" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I149">
@@ -35290,7 +35316,7 @@
       <c r="G150" t="s">
         <v>5</v>
       </c>
-      <c r="H150" s="2" t="s">
+      <c r="H150" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I150">
@@ -35454,7 +35480,7 @@
       <c r="G151" t="s">
         <v>3</v>
       </c>
-      <c r="H151" s="2" t="s">
+      <c r="H151" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I151">
@@ -35618,7 +35644,7 @@
       <c r="G152" t="s">
         <v>3</v>
       </c>
-      <c r="H152" s="2" t="s">
+      <c r="H152" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I152">
@@ -35782,7 +35808,7 @@
       <c r="G153" t="s">
         <v>3</v>
       </c>
-      <c r="H153" s="2" t="s">
+      <c r="H153" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I153">
@@ -35946,7 +35972,7 @@
       <c r="G154" t="s">
         <v>3</v>
       </c>
-      <c r="H154" s="1" t="s">
+      <c r="H154" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I154">
@@ -36110,7 +36136,7 @@
       <c r="G155" t="s">
         <v>5</v>
       </c>
-      <c r="H155" s="1" t="s">
+      <c r="H155" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I155">
@@ -36274,7 +36300,7 @@
       <c r="G156" t="s">
         <v>5</v>
       </c>
-      <c r="H156" s="2" t="s">
+      <c r="H156" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I156">
@@ -36438,7 +36464,7 @@
       <c r="G157" t="s">
         <v>5</v>
       </c>
-      <c r="H157" s="1" t="s">
+      <c r="H157" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I157">
@@ -36602,7 +36628,7 @@
       <c r="G158" t="s">
         <v>3</v>
       </c>
-      <c r="H158" s="2" t="s">
+      <c r="H158" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I158">
@@ -36766,7 +36792,7 @@
       <c r="G159" t="s">
         <v>5</v>
       </c>
-      <c r="H159" s="2" t="s">
+      <c r="H159" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I159">
@@ -36930,7 +36956,7 @@
       <c r="G160" t="s">
         <v>5</v>
       </c>
-      <c r="H160" s="1" t="s">
+      <c r="H160" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I160">
@@ -37094,7 +37120,7 @@
       <c r="G161" t="s">
         <v>3</v>
       </c>
-      <c r="H161" s="2" t="s">
+      <c r="H161" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I161">
@@ -37258,7 +37284,7 @@
       <c r="G162" t="s">
         <v>3</v>
       </c>
-      <c r="H162" s="2" t="s">
+      <c r="H162" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I162">
@@ -37422,7 +37448,7 @@
       <c r="G163" t="s">
         <v>3</v>
       </c>
-      <c r="H163" s="2" t="s">
+      <c r="H163" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I163">
@@ -37586,7 +37612,7 @@
       <c r="G164" t="s">
         <v>3</v>
       </c>
-      <c r="H164" s="2" t="s">
+      <c r="H164" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I164">
@@ -37750,7 +37776,7 @@
       <c r="G165" t="s">
         <v>3</v>
       </c>
-      <c r="H165" s="1" t="s">
+      <c r="H165" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I165">
@@ -37914,7 +37940,7 @@
       <c r="G166" t="s">
         <v>5</v>
       </c>
-      <c r="H166" s="2" t="s">
+      <c r="H166" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I166">
@@ -38078,7 +38104,7 @@
       <c r="G167" t="s">
         <v>3</v>
       </c>
-      <c r="H167" s="2" t="s">
+      <c r="H167" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I167">
@@ -38242,7 +38268,7 @@
       <c r="G168" t="s">
         <v>3</v>
       </c>
-      <c r="H168" s="2" t="s">
+      <c r="H168" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I168">
@@ -38406,7 +38432,7 @@
       <c r="G169" t="s">
         <v>5</v>
       </c>
-      <c r="H169" s="2" t="s">
+      <c r="H169" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I169">
@@ -38570,7 +38596,7 @@
       <c r="G170" t="s">
         <v>3</v>
       </c>
-      <c r="H170" s="2" t="s">
+      <c r="H170" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I170">
@@ -38734,7 +38760,7 @@
       <c r="G171" t="s">
         <v>3</v>
       </c>
-      <c r="H171" s="2" t="s">
+      <c r="H171" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I171">
@@ -38898,7 +38924,7 @@
       <c r="G172" t="s">
         <v>3</v>
       </c>
-      <c r="H172" s="2" t="s">
+      <c r="H172" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I172">
@@ -39062,7 +39088,7 @@
       <c r="G173" t="s">
         <v>5</v>
       </c>
-      <c r="H173" s="2" t="s">
+      <c r="H173" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I173">
@@ -39226,7 +39252,7 @@
       <c r="G174" t="s">
         <v>3</v>
       </c>
-      <c r="H174" s="2" t="s">
+      <c r="H174" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I174">
@@ -39390,7 +39416,7 @@
       <c r="G175" t="s">
         <v>5</v>
       </c>
-      <c r="H175" s="1" t="s">
+      <c r="H175" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I175">
@@ -39554,7 +39580,7 @@
       <c r="G176" t="s">
         <v>3</v>
       </c>
-      <c r="H176" s="2" t="s">
+      <c r="H176" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I176">
@@ -39718,7 +39744,7 @@
       <c r="G177" t="s">
         <v>3</v>
       </c>
-      <c r="H177" s="2" t="s">
+      <c r="H177" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I177">
@@ -39882,7 +39908,7 @@
       <c r="G178" t="s">
         <v>3</v>
       </c>
-      <c r="H178" s="2" t="s">
+      <c r="H178" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I178">
@@ -40046,7 +40072,7 @@
       <c r="G179" t="s">
         <v>5</v>
       </c>
-      <c r="H179" s="2" t="s">
+      <c r="H179" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I179">
@@ -40210,7 +40236,7 @@
       <c r="G180" t="s">
         <v>3</v>
       </c>
-      <c r="H180" s="2" t="s">
+      <c r="H180" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I180">
@@ -40374,7 +40400,7 @@
       <c r="G181" t="s">
         <v>3</v>
       </c>
-      <c r="H181" s="2" t="s">
+      <c r="H181" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I181">
@@ -40538,7 +40564,7 @@
       <c r="G182" t="s">
         <v>3</v>
       </c>
-      <c r="H182" s="1" t="s">
+      <c r="H182" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I182">
@@ -40702,7 +40728,7 @@
       <c r="G183" t="s">
         <v>3</v>
       </c>
-      <c r="H183" s="1" t="s">
+      <c r="H183" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I183">
@@ -40866,7 +40892,7 @@
       <c r="G184" t="s">
         <v>3</v>
       </c>
-      <c r="H184" s="1" t="s">
+      <c r="H184" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I184">
@@ -41030,7 +41056,7 @@
       <c r="G185" t="s">
         <v>5</v>
       </c>
-      <c r="H185" s="1" t="s">
+      <c r="H185" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I185">
@@ -41194,7 +41220,7 @@
       <c r="G186" t="s">
         <v>5</v>
       </c>
-      <c r="H186" s="1" t="s">
+      <c r="H186" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I186">
@@ -41358,7 +41384,7 @@
       <c r="G187" t="s">
         <v>5</v>
       </c>
-      <c r="H187" s="1" t="s">
+      <c r="H187" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I187">
@@ -41522,7 +41548,7 @@
       <c r="G188" t="s">
         <v>5</v>
       </c>
-      <c r="H188" s="2" t="s">
+      <c r="H188" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I188">
@@ -41686,7 +41712,7 @@
       <c r="G189" t="s">
         <v>5</v>
       </c>
-      <c r="H189" s="2" t="s">
+      <c r="H189" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I189">
@@ -41850,7 +41876,7 @@
       <c r="G190" t="s">
         <v>5</v>
       </c>
-      <c r="H190" s="1" t="s">
+      <c r="H190" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I190">
@@ -42014,7 +42040,7 @@
       <c r="G191" t="s">
         <v>5</v>
       </c>
-      <c r="H191" s="1" t="s">
+      <c r="H191" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I191">
@@ -42178,7 +42204,7 @@
       <c r="G192" t="s">
         <v>3</v>
       </c>
-      <c r="H192" s="2" t="s">
+      <c r="H192" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I192">
@@ -42342,7 +42368,7 @@
       <c r="G193" t="s">
         <v>3</v>
       </c>
-      <c r="H193" s="2" t="s">
+      <c r="H193" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I193">
@@ -42506,7 +42532,7 @@
       <c r="G194" t="s">
         <v>3</v>
       </c>
-      <c r="H194" s="2" t="s">
+      <c r="H194" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I194">
@@ -42670,7 +42696,7 @@
       <c r="G195" t="s">
         <v>5</v>
       </c>
-      <c r="H195" s="1" t="s">
+      <c r="H195" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I195">
@@ -42834,7 +42860,7 @@
       <c r="G196" t="s">
         <v>5</v>
       </c>
-      <c r="H196" s="2" t="s">
+      <c r="H196" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I196">
@@ -42998,7 +43024,7 @@
       <c r="G197" t="s">
         <v>5</v>
       </c>
-      <c r="H197" s="2" t="s">
+      <c r="H197" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I197">
@@ -43162,7 +43188,7 @@
       <c r="G198" t="s">
         <v>3</v>
       </c>
-      <c r="H198" s="2" t="s">
+      <c r="H198" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I198">
@@ -43326,7 +43352,7 @@
       <c r="G199" t="s">
         <v>3</v>
       </c>
-      <c r="H199" s="2" t="s">
+      <c r="H199" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I199">
@@ -43490,7 +43516,7 @@
       <c r="G200" t="s">
         <v>3</v>
       </c>
-      <c r="H200" s="2" t="s">
+      <c r="H200" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I200">
@@ -43654,7 +43680,7 @@
       <c r="G201" t="s">
         <v>3</v>
       </c>
-      <c r="H201" s="2" t="s">
+      <c r="H201" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I201">
@@ -43818,7 +43844,7 @@
       <c r="G202" t="s">
         <v>5</v>
       </c>
-      <c r="H202" s="1" t="s">
+      <c r="H202" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I202">
@@ -43982,7 +44008,7 @@
       <c r="G203" t="s">
         <v>5</v>
       </c>
-      <c r="H203" s="1" t="s">
+      <c r="H203" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I203">
@@ -44146,7 +44172,7 @@
       <c r="G204" t="s">
         <v>3</v>
       </c>
-      <c r="H204" s="2" t="s">
+      <c r="H204" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I204">
@@ -44310,7 +44336,7 @@
       <c r="G205" t="s">
         <v>5</v>
       </c>
-      <c r="H205" s="2" t="s">
+      <c r="H205" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I205">
@@ -44474,7 +44500,7 @@
       <c r="G206" t="s">
         <v>3</v>
       </c>
-      <c r="H206" s="2" t="s">
+      <c r="H206" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I206">
@@ -44638,7 +44664,7 @@
       <c r="G207" t="s">
         <v>3</v>
       </c>
-      <c r="H207" s="2" t="s">
+      <c r="H207" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I207">
@@ -44802,7 +44828,7 @@
       <c r="G208" t="s">
         <v>5</v>
       </c>
-      <c r="H208" s="1" t="s">
+      <c r="H208" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I208">
@@ -44966,7 +44992,7 @@
       <c r="G209" t="s">
         <v>3</v>
       </c>
-      <c r="H209" s="2" t="s">
+      <c r="H209" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I209">
@@ -45130,7 +45156,7 @@
       <c r="G210" t="s">
         <v>3</v>
       </c>
-      <c r="H210" s="1" t="s">
+      <c r="H210" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I210">
@@ -45294,7 +45320,7 @@
       <c r="G211" t="s">
         <v>3</v>
       </c>
-      <c r="H211" s="2" t="s">
+      <c r="H211" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I211">
@@ -45458,7 +45484,7 @@
       <c r="G212" t="s">
         <v>3</v>
       </c>
-      <c r="H212" s="2" t="s">
+      <c r="H212" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I212">
@@ -45622,7 +45648,7 @@
       <c r="G213" t="s">
         <v>3</v>
       </c>
-      <c r="H213" s="2" t="s">
+      <c r="H213" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I213">
@@ -45786,7 +45812,7 @@
       <c r="G214" t="s">
         <v>4</v>
       </c>
-      <c r="H214" s="1" t="s">
+      <c r="H214" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I214">
@@ -45950,7 +45976,7 @@
       <c r="G215" t="s">
         <v>3</v>
       </c>
-      <c r="H215" s="2" t="s">
+      <c r="H215" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I215">
@@ -46278,7 +46304,7 @@
       <c r="G217" t="s">
         <v>5</v>
       </c>
-      <c r="H217" s="2" t="s">
+      <c r="H217" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I217">
@@ -46442,7 +46468,7 @@
       <c r="G218" t="s">
         <v>5</v>
       </c>
-      <c r="H218" s="2" t="s">
+      <c r="H218" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I218">
@@ -46606,7 +46632,7 @@
       <c r="G219" t="s">
         <v>5</v>
       </c>
-      <c r="H219" s="1" t="s">
+      <c r="H219" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I219">
@@ -46770,7 +46796,7 @@
       <c r="G220" t="s">
         <v>5</v>
       </c>
-      <c r="H220" s="1" t="s">
+      <c r="H220" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I220">
@@ -46934,7 +46960,7 @@
       <c r="G221" t="s">
         <v>3</v>
       </c>
-      <c r="H221" s="2" t="s">
+      <c r="H221" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I221">
@@ -47098,7 +47124,7 @@
       <c r="G222" t="s">
         <v>3</v>
       </c>
-      <c r="H222" s="2" t="s">
+      <c r="H222" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I222">
@@ -47426,7 +47452,7 @@
       <c r="G224" t="s">
         <v>3</v>
       </c>
-      <c r="H224" s="2" t="s">
+      <c r="H224" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I224">
@@ -47590,7 +47616,7 @@
       <c r="G225" t="s">
         <v>5</v>
       </c>
-      <c r="H225" s="1" t="s">
+      <c r="H225" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I225">
@@ -47754,7 +47780,7 @@
       <c r="G226" t="s">
         <v>3</v>
       </c>
-      <c r="H226" s="2" t="s">
+      <c r="H226" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I226">
@@ -47918,7 +47944,7 @@
       <c r="G227" t="s">
         <v>3</v>
       </c>
-      <c r="H227" s="2" t="s">
+      <c r="H227" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I227">
@@ -48082,7 +48108,7 @@
       <c r="G228" t="s">
         <v>3</v>
       </c>
-      <c r="H228" s="2" t="s">
+      <c r="H228" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I228">
@@ -48246,7 +48272,7 @@
       <c r="G229" t="s">
         <v>3</v>
       </c>
-      <c r="H229" s="2" t="s">
+      <c r="H229" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I229">
@@ -48410,7 +48436,7 @@
       <c r="G230" t="s">
         <v>3</v>
       </c>
-      <c r="H230" s="2" t="s">
+      <c r="H230" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I230">
@@ -48574,7 +48600,7 @@
       <c r="G231" t="s">
         <v>5</v>
       </c>
-      <c r="H231" s="2" t="s">
+      <c r="H231" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I231">
@@ -48738,7 +48764,7 @@
       <c r="G232" t="s">
         <v>5</v>
       </c>
-      <c r="H232" s="2" t="s">
+      <c r="H232" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I232">
@@ -48902,7 +48928,7 @@
       <c r="G233" t="s">
         <v>3</v>
       </c>
-      <c r="H233" s="1" t="s">
+      <c r="H233" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I233">
@@ -49066,7 +49092,7 @@
       <c r="G234" t="s">
         <v>3</v>
       </c>
-      <c r="H234" s="2" t="s">
+      <c r="H234" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I234">
@@ -49230,7 +49256,7 @@
       <c r="G235" t="s">
         <v>3</v>
       </c>
-      <c r="H235" s="2" t="s">
+      <c r="H235" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I235">
@@ -49394,7 +49420,7 @@
       <c r="G236" t="s">
         <v>3</v>
       </c>
-      <c r="H236" s="2" t="s">
+      <c r="H236" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I236">
@@ -49558,7 +49584,7 @@
       <c r="G237" t="s">
         <v>5</v>
       </c>
-      <c r="H237" s="2" t="s">
+      <c r="H237" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I237">
@@ -49722,7 +49748,7 @@
       <c r="G238" t="s">
         <v>3</v>
       </c>
-      <c r="H238" s="1" t="s">
+      <c r="H238" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I238">
@@ -49886,7 +49912,7 @@
       <c r="G239" t="s">
         <v>3</v>
       </c>
-      <c r="H239" s="2" t="s">
+      <c r="H239" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I239">
@@ -50050,7 +50076,7 @@
       <c r="G240" t="s">
         <v>3</v>
       </c>
-      <c r="H240" s="2" t="s">
+      <c r="H240" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I240">
@@ -50214,7 +50240,7 @@
       <c r="G241" t="s">
         <v>3</v>
       </c>
-      <c r="H241" s="2" t="s">
+      <c r="H241" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I241">
@@ -50378,7 +50404,7 @@
       <c r="G242" t="s">
         <v>3</v>
       </c>
-      <c r="H242" s="2" t="s">
+      <c r="H242" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I242">
@@ -50542,7 +50568,7 @@
       <c r="G243" t="s">
         <v>3</v>
       </c>
-      <c r="H243" s="2" t="s">
+      <c r="H243" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I243">
@@ -50706,7 +50732,7 @@
       <c r="G244" t="s">
         <v>4</v>
       </c>
-      <c r="H244" s="1" t="s">
+      <c r="H244" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I244">
@@ -50870,7 +50896,7 @@
       <c r="G245" t="s">
         <v>3</v>
       </c>
-      <c r="H245" s="2" t="s">
+      <c r="H245" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I245">
@@ -51034,7 +51060,7 @@
       <c r="G246" t="s">
         <v>3</v>
       </c>
-      <c r="H246" s="2" t="s">
+      <c r="H246" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I246">
@@ -51198,7 +51224,7 @@
       <c r="G247" t="s">
         <v>5</v>
       </c>
-      <c r="H247" s="1" t="s">
+      <c r="H247" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I247">
@@ -51362,7 +51388,7 @@
       <c r="G248" t="s">
         <v>5</v>
       </c>
-      <c r="H248" s="1" t="s">
+      <c r="H248" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I248">
@@ -51526,7 +51552,7 @@
       <c r="G249" t="s">
         <v>5</v>
       </c>
-      <c r="H249" s="2" t="s">
+      <c r="H249" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I249">
@@ -51690,7 +51716,7 @@
       <c r="G250" t="s">
         <v>4</v>
       </c>
-      <c r="H250" s="1" t="s">
+      <c r="H250" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I250">
@@ -51854,7 +51880,7 @@
       <c r="G251" t="s">
         <v>5</v>
       </c>
-      <c r="H251" s="1" t="s">
+      <c r="H251" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I251">
@@ -52018,7 +52044,7 @@
       <c r="G252" t="s">
         <v>5</v>
       </c>
-      <c r="H252" s="1" t="s">
+      <c r="H252" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I252">
@@ -52182,7 +52208,7 @@
       <c r="G253" t="s">
         <v>5</v>
       </c>
-      <c r="H253" s="1" t="s">
+      <c r="H253" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I253">
@@ -52346,7 +52372,7 @@
       <c r="G254" t="s">
         <v>5</v>
       </c>
-      <c r="H254" s="2" t="s">
+      <c r="H254" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I254">
@@ -52510,7 +52536,7 @@
       <c r="G255" t="s">
         <v>5</v>
       </c>
-      <c r="H255" s="1" t="s">
+      <c r="H255" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I255">
@@ -52674,7 +52700,7 @@
       <c r="G256" t="s">
         <v>5</v>
       </c>
-      <c r="H256" s="2" t="s">
+      <c r="H256" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I256">
@@ -52838,7 +52864,7 @@
       <c r="G257" t="s">
         <v>3</v>
       </c>
-      <c r="H257" s="1" t="s">
+      <c r="H257" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I257">
@@ -53002,7 +53028,7 @@
       <c r="G258" t="s">
         <v>5</v>
       </c>
-      <c r="H258" s="2" t="s">
+      <c r="H258" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I258">
@@ -53166,7 +53192,7 @@
       <c r="G259" t="s">
         <v>3</v>
       </c>
-      <c r="H259" s="2" t="s">
+      <c r="H259" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I259">
@@ -53330,7 +53356,7 @@
       <c r="G260" t="s">
         <v>5</v>
       </c>
-      <c r="H260" s="2" t="s">
+      <c r="H260" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I260">
@@ -53494,7 +53520,7 @@
       <c r="G261" t="s">
         <v>5</v>
       </c>
-      <c r="H261" s="1" t="s">
+      <c r="H261" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I261">
@@ -53658,7 +53684,7 @@
       <c r="G262" t="s">
         <v>3</v>
       </c>
-      <c r="H262" s="2" t="s">
+      <c r="H262" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I262">
@@ -53822,7 +53848,7 @@
       <c r="G263" t="s">
         <v>3</v>
       </c>
-      <c r="H263" s="2" t="s">
+      <c r="H263" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I263">
@@ -53986,7 +54012,7 @@
       <c r="G264" t="s">
         <v>4</v>
       </c>
-      <c r="H264" s="1" t="s">
+      <c r="H264" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I264">
@@ -54150,7 +54176,7 @@
       <c r="G265" t="s">
         <v>3</v>
       </c>
-      <c r="H265" s="1" t="s">
+      <c r="H265" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I265">
@@ -54314,7 +54340,7 @@
       <c r="G266" t="s">
         <v>3</v>
       </c>
-      <c r="H266" s="2" t="s">
+      <c r="H266" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I266">
@@ -54478,7 +54504,7 @@
       <c r="G267" t="s">
         <v>3</v>
       </c>
-      <c r="H267" s="2" t="s">
+      <c r="H267" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I267">
@@ -54642,7 +54668,7 @@
       <c r="G268" t="s">
         <v>5</v>
       </c>
-      <c r="H268" s="1" t="s">
+      <c r="H268" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I268">
@@ -54806,7 +54832,7 @@
       <c r="G269" t="s">
         <v>3</v>
       </c>
-      <c r="H269" s="2" t="s">
+      <c r="H269" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I269">
@@ -54970,7 +54996,7 @@
       <c r="G270" t="s">
         <v>5</v>
       </c>
-      <c r="H270" s="1" t="s">
+      <c r="H270" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I270">
@@ -55298,7 +55324,7 @@
       <c r="G272" t="s">
         <v>3</v>
       </c>
-      <c r="H272" s="2" t="s">
+      <c r="H272" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I272">
@@ -55462,7 +55488,7 @@
       <c r="G273" t="s">
         <v>3</v>
       </c>
-      <c r="H273" s="1" t="s">
+      <c r="H273" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I273">
@@ -55626,7 +55652,7 @@
       <c r="G274" t="s">
         <v>5</v>
       </c>
-      <c r="H274" s="1" t="s">
+      <c r="H274" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I274">
@@ -55790,7 +55816,7 @@
       <c r="G275" t="s">
         <v>3</v>
       </c>
-      <c r="H275" s="1" t="s">
+      <c r="H275" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I275">
@@ -55954,7 +55980,7 @@
       <c r="G276" t="s">
         <v>3</v>
       </c>
-      <c r="H276" s="2" t="s">
+      <c r="H276" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I276">
@@ -56118,7 +56144,7 @@
       <c r="G277" t="s">
         <v>5</v>
       </c>
-      <c r="H277" s="1" t="s">
+      <c r="H277" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I277">
@@ -56282,7 +56308,7 @@
       <c r="G278" t="s">
         <v>5</v>
       </c>
-      <c r="H278" s="1" t="s">
+      <c r="H278" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I278">
@@ -56446,7 +56472,7 @@
       <c r="G279" t="s">
         <v>5</v>
       </c>
-      <c r="H279" s="1" t="s">
+      <c r="H279" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I279">
@@ -56610,7 +56636,7 @@
       <c r="G280" t="s">
         <v>5</v>
       </c>
-      <c r="H280" s="2" t="s">
+      <c r="H280" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I280">
@@ -56774,7 +56800,7 @@
       <c r="G281" t="s">
         <v>3</v>
       </c>
-      <c r="H281" s="1" t="s">
+      <c r="H281" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I281">
@@ -56938,7 +56964,7 @@
       <c r="G282" t="s">
         <v>5</v>
       </c>
-      <c r="H282" s="1" t="s">
+      <c r="H282" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I282">
@@ -57102,7 +57128,7 @@
       <c r="G283" t="s">
         <v>5</v>
       </c>
-      <c r="H283" s="1" t="s">
+      <c r="H283" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I283">
@@ -57266,7 +57292,7 @@
       <c r="G284" t="s">
         <v>3</v>
       </c>
-      <c r="H284" s="2" t="s">
+      <c r="H284" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I284">
@@ -57430,7 +57456,7 @@
       <c r="G285" t="s">
         <v>5</v>
       </c>
-      <c r="H285" s="1" t="s">
+      <c r="H285" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I285">
@@ -57594,7 +57620,7 @@
       <c r="G286" t="s">
         <v>3</v>
       </c>
-      <c r="H286" s="2" t="s">
+      <c r="H286" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I286">
@@ -57758,7 +57784,7 @@
       <c r="G287" t="s">
         <v>3</v>
       </c>
-      <c r="H287" s="2" t="s">
+      <c r="H287" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I287">
@@ -57922,7 +57948,7 @@
       <c r="G288" t="s">
         <v>4</v>
       </c>
-      <c r="H288" s="1" t="s">
+      <c r="H288" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I288">
@@ -58086,7 +58112,7 @@
       <c r="G289" t="s">
         <v>3</v>
       </c>
-      <c r="H289" s="2" t="s">
+      <c r="H289" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I289">
@@ -58250,7 +58276,7 @@
       <c r="G290" t="s">
         <v>3</v>
       </c>
-      <c r="H290" s="2" t="s">
+      <c r="H290" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I290">
@@ -58414,7 +58440,7 @@
       <c r="G291" t="s">
         <v>3</v>
       </c>
-      <c r="H291" s="2" t="s">
+      <c r="H291" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I291">
@@ -58578,7 +58604,7 @@
       <c r="G292" t="s">
         <v>5</v>
       </c>
-      <c r="H292" s="1" t="s">
+      <c r="H292" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I292">
@@ -58742,7 +58768,7 @@
       <c r="G293" t="s">
         <v>5</v>
       </c>
-      <c r="H293" s="1" t="s">
+      <c r="H293" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I293">
@@ -58906,7 +58932,7 @@
       <c r="G294" t="s">
         <v>5</v>
       </c>
-      <c r="H294" s="2" t="s">
+      <c r="H294" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I294">
@@ -59070,7 +59096,7 @@
       <c r="G295" t="s">
         <v>3</v>
       </c>
-      <c r="H295" s="2" t="s">
+      <c r="H295" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I295">
@@ -59234,7 +59260,7 @@
       <c r="G296" t="s">
         <v>3</v>
       </c>
-      <c r="H296" s="2" t="s">
+      <c r="H296" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I296">
@@ -59398,7 +59424,7 @@
       <c r="G297" t="s">
         <v>3</v>
       </c>
-      <c r="H297" s="1" t="s">
+      <c r="H297" s="2" t="s">
         <v>933</v>
       </c>
       <c r="I297">
@@ -59562,7 +59588,7 @@
       <c r="G298" t="s">
         <v>3</v>
       </c>
-      <c r="H298" s="2" t="s">
+      <c r="H298" s="3" t="s">
         <v>934</v>
       </c>
       <c r="I298">
@@ -59726,7 +59752,7 @@
       <c r="G299" t="s">
         <v>5</v>
       </c>
-      <c r="H299" s="1" t="s">
+      <c r="H299" s="2" t="s">
         <v>934</v>
       </c>
       <c r="I299">
@@ -59890,7 +59916,7 @@
       <c r="G300" t="s">
         <v>5</v>
       </c>
-      <c r="H300" s="2" t="s">
+      <c r="H300" s="3" t="s">
         <v>933</v>
       </c>
       <c r="I300">
@@ -60048,22 +60074,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>937</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>938</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>939</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>940</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>941</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>942</v>
       </c>
     </row>

</xml_diff>